<commit_message>
Clasificación G2: el motor no nombra ninguna familia
- Detección genérica: implicaciones de palabras clave, ámbitos que dejan de
  aplicar, evidencia del uso sobre valores por defecto y nueva deducción de
  atributos dependientes; patrones sobre cualquier parte de la composición.
- Lectura de la composición según los atributos que derivan de cada parte;
  modos «superficie» y «contacto»; partes informativas por dato.
- Frases «PARA HOMBRE/NIÑA/UNISEX…» y vocabulario de materiales como datos.
- Dominio de cada categoría en los datos; ficha genérica para productos sin
  familia. Migración 0025. Prueba que vigila que el motor no nombre familias.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Grf21aTokQ4uAJp8cAKh7e
</commit_message>
<xml_diff>
--- a/backend/app/data/motor/02_carga_motor_dinamico_v3.xlsx
+++ b/backend/app/data/motor/02_carga_motor_dinamico_v3.xlsx
@@ -2501,7 +2501,7 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>Only for products without a configured category: their own technical sheet asks what matters.</t>
+          <t>Only for products outside a configured family (no domain): a family's own technical sheet asks what matters.</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>dominio</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
Catálogo de las Notas Explicativas conectado: migración 0034, semilla por familia y pruebas
- Semilla por familia (calzado, ropa, accesorios, químicos, materias primas) que
  leen atributos, categorías, reglas, clases de material y dominios.
- Migración 0034: borra la configuración anterior del motor y mapea categorías.
- Valores por defecto solo de las preguntas de la categoría; no se guardan los
  de preguntas ajenas. La materia que nombra el producto se sugiere primero.
- Datos nacionales con ámbito en ropa y calzado; partes de calzado no se
  confunden con un calzado completo que describe su corte y suela.
- Pruebas actualizadas a los códigos nuevos y casos de las Notas por familia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Grf21aTokQ4uAJp8cAKh7e
</commit_message>
<xml_diff>
--- a/backend/app/data/motor/02_carga_motor_dinamico_v3.xlsx
+++ b/backend/app/data/motor/02_carga_motor_dinamico_v3.xlsx
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -971,141 +971,6 @@
       <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Default mode</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>Chemicals</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>Chemical substances, mixtures and chemical preparations; dynamic questions based on remaining candidates.</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Raw materials</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Materials and semi-processed inputs across multiple chapters; never treated as a single tariff chapter.</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>FOOTWEAR</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Footwear</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Footwear and directly related constructions/material distinctions.</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>APPAREL</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Apparel</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Garments and textile clothing; includes knitted/woven and fiber composition logic.</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>ACCESSORIES_MERCH</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Accessories / merchandise</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Brand merchandise and daily-use accessories: bags, headwear, pins, bottle openers, boards/sport articles, holders, straps and similar; open-ended.</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>AUTO</t>
         </is>
       </c>
     </row>
@@ -1123,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1184,118 +1049,116 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Product / commercial name</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Short product name; used for search/candidate generation only.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>technical_description</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Technical description</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Technical description sufficient to distinguish construction, composition and function.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>material_composition</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Material composition</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>composition</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Multiple materials and percentages.</t>
         </is>
@@ -1307,660 +1170,229 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>manufacturing_process</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Manufacturing / processing process</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>multi_select</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Processes only when relevant to candidate distinction.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>presentation_form</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Presentation / physical form</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>select</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Bulk, retail pack, sheet, roll, finished article, set, part, etc.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>intended_use</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Intended use</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Use only when legally or technically relevant.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>complete_or_incomplete</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Complete / incomplete</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>select</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Supports GRI workflow when article is incomplete or unfinished.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>dimensions</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Dimensions</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>measurement_set</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Capture only if candidate rules require size/measurements.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>net_weight</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Net weight</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>CORE</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Use only when thresholds or headings depend on weight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>substance_or_mixture</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Substance or mixture</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>select</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Distinguish single substance vs mixture/preparation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>chemical_name</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Chemical / technical name</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Technical identification when known.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>cas_number</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>CAS number</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Optional identifier; never required if unavailable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Physical state</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>select</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Solid, liquid, gas, powder, paste, etc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>concentration</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Concentration</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Relevant percentage when classification depends on concentration/composition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>purity</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Purity</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Relevant when legal text distinguishes purity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>chemical_function</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Chemical function / use</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Functional description if the tariff distinction depends on use/preparation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>processing_degree</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Processing degree</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>select</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>Raw, semi-processed, finished, coated, treated, etc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>material_grade</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Material grade/specification</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Only when the tariff rule distinguishes grade/specification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>shape_form</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Shape / form</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>select</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>Sheet, bar, roll, granule, powder, profile, yarn, fabric, etc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>coating_treatment</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Coating / treatment</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>multi_select</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>Relevant treatments/coatings.</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2022,360 +1454,60 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>SOLID</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>solid</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>complete_or_incomplete</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>LIQUID</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Liquid</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>liquid</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>complete_or_incomplete</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>unfinished</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>20</v>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>GAS</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Gas</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>gas</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>POWDER</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Powder</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>powder</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>PASTE</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Paste / gel</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>paste; gel</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>substance_or_mixture</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>SUBSTANCE</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Single substance</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>pure substance; compound</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>substance_or_mixture</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>MIXTURE</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Mixture / preparation</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>mixture; preparation; formulation</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>complete_or_incomplete</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>complete_or_incomplete</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Incomplete</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>unfinished</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>processing_degree</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>RAW</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>Raw / unprocessed</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>processing_degree</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>SEMI_PROCESSED</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Semi-processed</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>intermediate; semi finished</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>processing_degree</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>FINISHED</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>Finished material/article</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2395,7 +1527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2445,346 +1577,65 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>REQUIRE</t>
         </is>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" t="n">
         <v>1000</v>
       </c>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>technical_description</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>SHOW</t>
         </is>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" t="n">
         <v>900</v>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Only for products outside a configured family (no domain): a family's own technical sheet asks what matters.</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>substance_or_mixture</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="n">
-        <v>900</v>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Show when chemical candidates remain.</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>chemical_name</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>850</v>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Optional if technical identity is known.</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>cas_number</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Optional helper identifier.</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>physical_state</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>800</v>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Show only when candidate rules use state/form.</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>concentration</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>700</v>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Ask when threshold/composition matters.</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>purity</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>CHEMICALS</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>650</v>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Ask when legal distinction depends on purity.</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>processing_degree</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>900</v>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Common discriminator for raw vs semi-processed material.</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>shape_form</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>RAW_MATERIALS</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>SHOW</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>850</v>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Show if form/shape affects candidates.</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>